<commit_message>
put parcel_value variable in functions and also in excels for zero cod booking
</commit_message>
<xml_diff>
--- a/public/file/Trax Book Corporate Omni Shipment Template.xlsx
+++ b/public/file/Trax Book Corporate Omni Shipment Template.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26130"/>
+  <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\sonic\public\file\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BF430CC-91CD-4B6E-8245-F9FE58904EF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1884" yWindow="1884" windowWidth="17280" windowHeight="8964"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -24,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="33">
   <si>
     <t>Consignee Name</t>
   </si>
@@ -120,12 +121,15 @@
   </si>
   <si>
     <t>Return Address Id</t>
+  </si>
+  <si>
+    <t>Parcel Value</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -471,8 +475,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AF1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:AG1"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15.33203125" style="1" bestFit="1" customWidth="1"/>
@@ -503,7 +507,7 @@
     <col min="31" max="31" width="16.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>7</v>
       </c>
@@ -599,6 +603,9 @@
       </c>
       <c r="AF1" s="1" t="s">
         <v>31</v>
+      </c>
+      <c r="AG1" s="1" t="s">
+        <v>32</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
worked on zero cod parcel value
</commit_message>
<xml_diff>
--- a/public/file/Trax Book Corporate Omni Shipment Template.xlsx
+++ b/public/file/Trax Book Corporate Omni Shipment Template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\sonic\public\file\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BF430CC-91CD-4B6E-8245-F9FE58904EF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9616B1D-EBA3-4B25-B11E-4CB7ABEA847A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2544" yWindow="2544" windowWidth="17280" windowHeight="8964" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
first mile work done excel booking work done and reverse pickup handle
</commit_message>
<xml_diff>
--- a/public/file/Trax Book Corporate Omni Shipment Template.xlsx
+++ b/public/file/Trax Book Corporate Omni Shipment Template.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="37">
   <si>
     <t>Consignee Name</t>
   </si>
@@ -129,6 +129,12 @@
   </si>
   <si>
     <t>Consignee Address Longitude</t>
+  </si>
+  <si>
+    <t>Retail Pickup Store ID</t>
+  </si>
+  <si>
+    <t>Retail Deliver Store ID</t>
   </si>
 </sst>
 </file>
@@ -481,7 +487,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AI1"/>
+  <dimension ref="A1:AK1"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15.33203125" style="1" bestFit="1" customWidth="1"/>
@@ -512,7 +518,7 @@
     <col min="33" max="33" width="16.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:35" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:37" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>7</v>
       </c>
@@ -617,6 +623,12 @@
       </c>
       <c r="AI1" s="1" t="s">
         <v>32</v>
+      </c>
+      <c r="AJ1" t="s">
+        <v>35</v>
+      </c>
+      <c r="AK1" t="s">
+        <v>36</v>
       </c>
     </row>
   </sheetData>

</xml_diff>